<commit_message>
v0.4.1 - ISA withdrawals integrated into retirement strategy
</commit_message>
<xml_diff>
--- a/RetirementPlanner.xlsx
+++ b/RetirementPlanner.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Charts" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Assumptions'!$A$1:$B$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Assumptions'!$A$1:$B$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Cash Flow'!$A$1:$M$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -483,7 +483,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>1926291.01</v>
+        <v>1374378.42</v>
       </c>
     </row>
     <row r="7">
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>955244.29</v>
+        <v>149935.17</v>
       </c>
     </row>
     <row r="8">
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>0</v>
+        <v>25167.22</v>
       </c>
     </row>
     <row r="9">
@@ -513,7 +513,7 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>955244.29</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B37"/>
+  <dimension ref="A1:B38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -589,37 +589,37 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>starting_pension</t>
+          <t>max_pension_income</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>660000</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>expected_investment_return</t>
+          <t>starting_pension</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.0475</v>
+        <v>660000</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>platform_charge</t>
+          <t>expected_investment_return</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.0025</v>
+        <v>0.0475</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>fund_charge</t>
+          <t>platform_charge</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -629,267 +629,267 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>target_net_income</t>
+          <t>fund_charge</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>35000</v>
+        <v>0.0025</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>starting_savings</t>
+          <t>target_net_income</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>11000</v>
+        <v>35000</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>savings_interest_rate</t>
+          <t>starting_savings</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.03</v>
+        <v>11000</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>inflation</t>
+          <t>savings_interest_rate</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.025</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>personal_allowance</t>
+          <t>inflation</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>12570</v>
+        <v>0.025</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>basic_rate_limit</t>
+          <t>personal_allowance</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>50270</v>
+        <v>12570</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>basic_rate</t>
+          <t>basic_rate_limit</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.2</v>
+        <v>50270</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>higher_rate</t>
+          <t>basic_rate</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>additional_rate</t>
+          <t>higher_rate</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.45</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>pension_growth</t>
+          <t>additional_rate</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.04</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>savings_interest</t>
+          <t>pension_growth</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.035</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>starting_isa</t>
+          <t>savings_interest</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>50000</v>
+        <v>0.035</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>isa_growth_rate</t>
+          <t>starting_isa</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.04</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>annual_isa_allowance</t>
+          <t>isa_growth_rate</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>40000</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>property_sale</t>
+          <t>annual_isa_allowance</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>350000</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>property_sale_age</t>
+          <t>property_sale</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>67</v>
+        <v>350000</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>state_pension_full</t>
+          <t>property_sale_age</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>12548</v>
+        <v>67</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>current_calendar_year</t>
+          <t>state_pension_full</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2026</v>
+        <v>12548</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>state_pension_growth</t>
+          <t>current_calendar_year</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>0.035</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>spending_phase_1</t>
+          <t>state_pension_growth</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>35000</v>
+        <v>0.035</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>spending_phase_2</t>
+          <t>spending_phase_1</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>32000</v>
+        <v>35000</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>spending_phase_3</t>
+          <t>spending_phase_2</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>28000</v>
+        <v>32000</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>phase_1_end_age</t>
+          <t>spending_phase_3</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>69</v>
+        <v>28000</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>phase_2_end_age</t>
+          <t>phase_1_end_age</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>79</v>
+        <v>69</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>inflation_rate</t>
+          <t>phase_2_end_age</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>0.025</v>
+        <v>79</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>inflation_link_spending</t>
-        </is>
-      </c>
-      <c r="B35" t="b">
-        <v>1</v>
+          <t>inflation_rate</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>0.025</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>inflation_link_tax</t>
+          <t>inflation_link_spending</t>
         </is>
       </c>
       <c r="B36" t="b">
@@ -899,15 +899,25 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>inflation_link_isa</t>
+          <t>inflation_link_tax</t>
         </is>
       </c>
       <c r="B37" t="b">
         <v>1</v>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>inflation_link_isa</t>
+        </is>
+      </c>
+      <c r="B38" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B37"/>
+  <autoFilter ref="A1:B38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -931,7 +941,7 @@
     <col width="21" customWidth="1" min="8" max="8"/>
     <col width="23" customWidth="1" min="9" max="9"/>
     <col width="17" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="15" customWidth="1" min="13" max="13"/>
   </cols>
@@ -1017,13 +1027,13 @@
         <v>26400</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0</v>
+        <v>34357.5</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0</v>
+        <v>4357.5</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>0</v>
@@ -1035,10 +1045,10 @@
         <v>330</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>0</v>
+        <v>11330</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>63330</v>
+        <v>52000</v>
       </c>
       <c r="M2" s="2" t="n">
         <v>0</v>
@@ -1052,19 +1062,19 @@
         <v>2028</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>686400</v>
+        <v>652042.5</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>27456</v>
+        <v>26081.7</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0</v>
+        <v>34357.5</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0</v>
+        <v>4357.5</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>0</v>
@@ -1076,10 +1086,10 @@
         <v>339.9</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>0</v>
+        <v>11669.9</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>77533.10000000001</v>
+        <v>54080</v>
       </c>
       <c r="M3" s="2" t="n">
         <v>0</v>
@@ -1093,19 +1103,19 @@
         <v>2029</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>713856</v>
+        <v>643766.7</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>28554.24</v>
+        <v>25750.67</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0</v>
+        <v>34357.5</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0</v>
+        <v>4357.5</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>0</v>
@@ -1117,10 +1127,10 @@
         <v>350.1</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>0</v>
+        <v>12020</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>92654.42</v>
+        <v>56243.2</v>
       </c>
       <c r="M4" s="2" t="n">
         <v>0</v>
@@ -1134,19 +1144,19 @@
         <v>2030</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>742410.24</v>
+        <v>635159.87</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>29696.41</v>
+        <v>25406.39</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0</v>
+        <v>34357.5</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0</v>
+        <v>4357.5</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>0</v>
@@ -1158,10 +1168,10 @@
         <v>360.6</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>0</v>
+        <v>12380.6</v>
       </c>
       <c r="L5" s="2" t="n">
-        <v>108741.2</v>
+        <v>58492.93</v>
       </c>
       <c r="M5" s="2" t="n">
         <v>0</v>
@@ -1175,19 +1185,19 @@
         <v>2031</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>772106.65</v>
+        <v>626208.76</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>30884.27</v>
+        <v>25048.35</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>0</v>
+        <v>27595.22</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0</v>
+        <v>5514.64</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0</v>
+        <v>22080.58</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>12548</v>
@@ -1199,10 +1209,10 @@
         <v>12919.42</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>0</v>
+        <v>12752.02</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>125842.87</v>
+        <v>60832.65</v>
       </c>
       <c r="M6" s="2" t="n">
         <v>0</v>
@@ -1216,19 +1226,19 @@
         <v>2032</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>802990.92</v>
+        <v>623661.89</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>32119.64</v>
+        <v>24946.48</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>104.29</v>
+        <v>27142.12</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>104.29</v>
+        <v>5511.86</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>0</v>
+        <v>21630.26</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>12987.18</v>
@@ -1240,10 +1250,10 @@
         <v>13369.74</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>0</v>
+        <v>13134.58</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>144011.16</v>
+        <v>63265.95</v>
       </c>
       <c r="M7" s="2" t="n">
         <v>0</v>
@@ -1257,19 +1267,19 @@
         <v>2033</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>835006.26</v>
+        <v>621466.25</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>33400.25</v>
+        <v>24858.65</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>217.93</v>
+        <v>9871.059999999999</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>217.93</v>
+        <v>2148.56</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>0</v>
+        <v>7722.5</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>13441.73</v>
@@ -1281,10 +1291,10 @@
         <v>27277.5</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>0</v>
+        <v>13528.62</v>
       </c>
       <c r="L8" s="2" t="n">
-        <v>163300.23</v>
+        <v>65796.59</v>
       </c>
       <c r="M8" s="2" t="n">
         <v>0</v>
@@ -1298,19 +1308,19 @@
         <v>2034</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>868188.58</v>
+        <v>636453.84</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>34727.54</v>
+        <v>25458.15</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>335.55</v>
+        <v>5047.75</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>335.55</v>
+        <v>1277.99</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>0</v>
+        <v>3769.76</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>13912.19</v>
@@ -1322,10 +1332,10 @@
         <v>28230.24</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>0</v>
+        <v>13934.48</v>
       </c>
       <c r="L9" s="2" t="n">
-        <v>183766.72</v>
+        <v>68428.45</v>
       </c>
       <c r="M9" s="2" t="n">
         <v>0</v>
@@ -1339,19 +1349,19 @@
         <v>2035</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>902580.58</v>
+        <v>656864.24</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>36103.22</v>
+        <v>26274.57</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>457.28</v>
+        <v>3936.94</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>457.28</v>
+        <v>1153.21</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>0</v>
+        <v>2783.73</v>
       </c>
       <c r="H10" s="2" t="n">
         <v>14399.12</v>
@@ -1363,10 +1373,10 @@
         <v>29216.27</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>0</v>
+        <v>14352.51</v>
       </c>
       <c r="L10" s="2" t="n">
-        <v>205469.9</v>
+        <v>71165.59</v>
       </c>
       <c r="M10" s="2" t="n">
         <v>0</v>
@@ -1380,19 +1390,19 @@
         <v>2036</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>938226.52</v>
+        <v>679201.87</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>37529.06</v>
+        <v>27168.07</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>583.27</v>
+        <v>2787.32</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>583.27</v>
+        <v>1024.08</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>0</v>
+        <v>1763.24</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>14903.09</v>
@@ -1404,10 +1414,10 @@
         <v>30236.76</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>0</v>
+        <v>14783.09</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>228471.78</v>
+        <v>74012.21000000001</v>
       </c>
       <c r="M11" s="2" t="n">
         <v>0</v>
@@ -1421,19 +1431,19 @@
         <v>2037</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>975172.3100000001</v>
+        <v>703582.63</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>39006.89</v>
+        <v>28143.31</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>713.67</v>
+        <v>1597.56</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>713.67</v>
+        <v>890.45</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>0</v>
+        <v>707.11</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>15424.7</v>
@@ -1445,10 +1455,10 @@
         <v>31292.89</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>0</v>
+        <v>15226.58</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>252837.24</v>
+        <v>76972.7</v>
       </c>
       <c r="M12" s="2" t="n">
         <v>0</v>
@@ -1462,10 +1472,10 @@
         <v>2038</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>1013465.53</v>
+        <v>730128.37</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>40538.62</v>
+        <v>29205.13</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>848.64</v>
@@ -1486,10 +1496,10 @@
         <v>32385.92</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>0</v>
+        <v>15683.38</v>
       </c>
       <c r="L13" s="2" t="n">
-        <v>278634.11</v>
+        <v>80051.61</v>
       </c>
       <c r="M13" s="2" t="n">
         <v>0</v>
@@ -1503,10 +1513,10 @@
         <v>2039</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>1053155.51</v>
+        <v>758484.87</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>42126.22</v>
+        <v>30339.39</v>
       </c>
       <c r="E14" s="2" t="n">
         <v>988.33</v>
@@ -1527,10 +1537,10 @@
         <v>33517.14</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>0</v>
+        <v>16153.88</v>
       </c>
       <c r="L14" s="2" t="n">
-        <v>305933.35</v>
+        <v>83253.67999999999</v>
       </c>
       <c r="M14" s="2" t="n">
         <v>0</v>
@@ -1544,10 +1554,10 @@
         <v>2040</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>1094293.4</v>
+        <v>787835.9300000001</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>43771.74</v>
+        <v>31513.44</v>
       </c>
       <c r="E15" s="2" t="n">
         <v>1132.91</v>
@@ -1568,10 +1578,10 @@
         <v>34687.9</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>0</v>
+        <v>16638.5</v>
       </c>
       <c r="L15" s="2" t="n">
-        <v>334809.18</v>
+        <v>86583.82000000001</v>
       </c>
       <c r="M15" s="2" t="n">
         <v>0</v>
@@ -1585,10 +1595,10 @@
         <v>2041</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1136932.23</v>
+        <v>818216.46</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>45477.29</v>
+        <v>32728.66</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>1282.55</v>
@@ -1609,10 +1619,10 @@
         <v>35899.53</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>0</v>
+        <v>17137.65</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>365339.2</v>
+        <v>90047.17999999999</v>
       </c>
       <c r="M16" s="2" t="n">
         <v>0</v>
@@ -1626,10 +1636,10 @@
         <v>2042</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>1181126.97</v>
+        <v>849662.5699999999</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>47245.08</v>
+        <v>33986.5</v>
       </c>
       <c r="E17" s="2" t="n">
         <v>1437.42</v>
@@ -1650,10 +1660,10 @@
         <v>37153.53</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>0</v>
+        <v>17651.78</v>
       </c>
       <c r="L17" s="2" t="n">
-        <v>397604.55</v>
+        <v>93649.06</v>
       </c>
       <c r="M17" s="2" t="n">
         <v>0</v>
@@ -1667,10 +1677,10 @@
         <v>2043</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1226934.63</v>
+        <v>882211.65</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>49077.39</v>
+        <v>35288.47</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>1597.72</v>
@@ -1691,10 +1701,10 @@
         <v>38451.33</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>0</v>
+        <v>18181.33</v>
       </c>
       <c r="L18" s="2" t="n">
-        <v>431690.06</v>
+        <v>97395.02</v>
       </c>
       <c r="M18" s="2" t="n">
         <v>0</v>
@@ -1708,10 +1718,10 @@
         <v>2044</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1274414.29</v>
+        <v>915902.4</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>50976.57</v>
+        <v>36636.1</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>1763.63</v>
@@ -1732,10 +1742,10 @@
         <v>39794.48</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>0</v>
+        <v>18726.77</v>
       </c>
       <c r="L19" s="2" t="n">
-        <v>467684.43</v>
+        <v>101290.83</v>
       </c>
       <c r="M19" s="2" t="n">
         <v>0</v>
@@ -1749,10 +1759,10 @@
         <v>2045</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1323627.24</v>
+        <v>950774.86</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>52945.09</v>
+        <v>38030.99</v>
       </c>
       <c r="E20" s="2" t="n">
         <v>1935.34</v>
@@ -1773,10 +1783,10 @@
         <v>41184.56</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>0</v>
+        <v>19288.57</v>
       </c>
       <c r="L20" s="2" t="n">
-        <v>505680.38</v>
+        <v>105342.46</v>
       </c>
       <c r="M20" s="2" t="n">
         <v>0</v>
@@ -1790,10 +1800,10 @@
         <v>2046</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1374636.98</v>
+        <v>986870.52</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>54985.48</v>
+        <v>39474.82</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>2113.07</v>
@@ -1814,10 +1824,10 @@
         <v>42623.22</v>
       </c>
       <c r="K21" s="2" t="n">
-        <v>0</v>
+        <v>19867.23</v>
       </c>
       <c r="L21" s="2" t="n">
-        <v>545774.83</v>
+        <v>109556.16</v>
       </c>
       <c r="M21" s="2" t="n">
         <v>0</v>
@@ -1831,10 +1841,10 @@
         <v>2047</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1427509.39</v>
+        <v>1024232.27</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>57100.38</v>
+        <v>40969.29</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>2297.01</v>
@@ -1855,10 +1865,10 @@
         <v>44112.14</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>0</v>
+        <v>20463.25</v>
       </c>
       <c r="L22" s="2" t="n">
-        <v>588069.0699999999</v>
+        <v>113938.4</v>
       </c>
       <c r="M22" s="2" t="n">
         <v>0</v>
@@ -1872,10 +1882,10 @@
         <v>2048</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>1482312.76</v>
+        <v>1062904.55</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>59292.51</v>
+        <v>42516.18</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>2487.4</v>
@@ -1896,10 +1906,10 @@
         <v>45653.08</v>
       </c>
       <c r="K23" s="2" t="n">
-        <v>0</v>
+        <v>21077.15</v>
       </c>
       <c r="L23" s="2" t="n">
-        <v>632668.98</v>
+        <v>118495.94</v>
       </c>
       <c r="M23" s="2" t="n">
         <v>0</v>
@@ -1913,10 +1923,10 @@
         <v>2049</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1539117.87</v>
+        <v>1102933.33</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>61564.71</v>
+        <v>44117.33</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>2684.44</v>
@@ -1937,10 +1947,10 @@
         <v>47247.85</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>0</v>
+        <v>21709.46</v>
       </c>
       <c r="L24" s="2" t="n">
-        <v>679685.2</v>
+        <v>123235.78</v>
       </c>
       <c r="M24" s="2" t="n">
         <v>0</v>
@@ -1954,10 +1964,10 @@
         <v>2050</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>1597998.14</v>
+        <v>1144366.22</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>63919.93</v>
+        <v>45774.65</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>2888.39</v>
@@ -1978,10 +1988,10 @@
         <v>48898.38</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>0</v>
+        <v>22360.74</v>
       </c>
       <c r="L25" s="2" t="n">
-        <v>729233.35</v>
+        <v>128165.21</v>
       </c>
       <c r="M25" s="2" t="n">
         <v>0</v>
@@ -1995,10 +2005,10 @@
         <v>2051</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>1659029.68</v>
+        <v>1187252.48</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>66361.19</v>
+        <v>47490.1</v>
       </c>
       <c r="E26" s="2" t="n">
         <v>3099.47</v>
@@ -2019,10 +2029,10 @@
         <v>50606.56</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>0</v>
+        <v>23031.56</v>
       </c>
       <c r="L26" s="2" t="n">
-        <v>781434.24</v>
+        <v>133291.82</v>
       </c>
       <c r="M26" s="2" t="n">
         <v>0</v>
@@ -2036,10 +2046,10 @@
         <v>2052</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>1722291.4</v>
+        <v>1231643.11</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>68891.66</v>
+        <v>49265.72</v>
       </c>
       <c r="E27" s="2" t="n">
         <v>3317.94</v>
@@ -2060,10 +2070,10 @@
         <v>52374.45</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>0</v>
+        <v>23722.51</v>
       </c>
       <c r="L27" s="2" t="n">
-        <v>836414.12</v>
+        <v>138623.49</v>
       </c>
       <c r="M27" s="2" t="n">
         <v>0</v>
@@ -2077,10 +2087,10 @@
         <v>2053</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>1787865.11</v>
+        <v>1277590.9</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>71514.60000000001</v>
+        <v>51103.64</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>3544.05</v>
@@ -2101,10 +2111,10 @@
         <v>54204.1</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>0</v>
+        <v>24434.19</v>
       </c>
       <c r="L28" s="2" t="n">
-        <v>894304.88</v>
+        <v>144168.43</v>
       </c>
       <c r="M28" s="2" t="n">
         <v>0</v>
@@ -2118,10 +2128,10 @@
         <v>2054</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>1855835.67</v>
+        <v>1325150.48</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>74233.42999999999</v>
+        <v>53006.02</v>
       </c>
       <c r="E29" s="2" t="n">
         <v>3778.08</v>
@@ -2142,13 +2152,13 @@
         <v>56097.67</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>0</v>
+        <v>25167.22</v>
       </c>
       <c r="L29" s="2" t="n">
-        <v>955244.29</v>
+        <v>149935.17</v>
       </c>
       <c r="M29" s="2" t="n">
-        <v>955244.29</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v0.5.0 - Retirement planning engine with configurable withdrawal strategies
</commit_message>
<xml_diff>
--- a/RetirementPlanner.xlsx
+++ b/RetirementPlanner.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Charts" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Assumptions'!$A$1:$B$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Assumptions'!$A$1:$B$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Cash Flow'!$A$1:$M$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -483,7 +483,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>1374378.42</v>
+        <v>1311036.72</v>
       </c>
     </row>
     <row r="7">
@@ -527,11 +527,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B38"/>
+  <dimension ref="A1:B39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -549,87 +549,89 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>current_age</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>62</v>
+          <t>withdrawal_strategy</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>PENSION_FIRST</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>retirement_age</t>
+          <t>current_age</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>projection_end_age</t>
+          <t>retirement_age</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>90</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>spouse_current_age</t>
+          <t>projection_end_age</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>59</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>max_pension_income</t>
+          <t>spouse_current_age</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>30000</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>starting_pension</t>
+          <t>max_pension_income</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>660000</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>expected_investment_return</t>
+          <t>starting_pension</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.0475</v>
+        <v>660000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>platform_charge</t>
+          <t>expected_investment_return</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.0025</v>
+        <v>0.0475</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>fund_charge</t>
+          <t>platform_charge</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -639,267 +641,267 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>target_net_income</t>
+          <t>fund_charge</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>35000</v>
+        <v>0.0025</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>starting_savings</t>
+          <t>target_net_income</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>11000</v>
+        <v>35000</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>savings_interest_rate</t>
+          <t>starting_savings</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.03</v>
+        <v>11000</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>inflation</t>
+          <t>savings_interest_rate</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.025</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>personal_allowance</t>
+          <t>inflation</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>12570</v>
+        <v>0.025</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>basic_rate_limit</t>
+          <t>personal_allowance</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>50270</v>
+        <v>12570</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>basic_rate</t>
+          <t>basic_rate_limit</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.2</v>
+        <v>50270</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>higher_rate</t>
+          <t>basic_rate</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>additional_rate</t>
+          <t>higher_rate</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.45</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>pension_growth</t>
+          <t>additional_rate</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.04</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>savings_interest</t>
+          <t>pension_growth</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.035</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>starting_isa</t>
+          <t>savings_interest</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>50000</v>
+        <v>0.035</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>isa_growth_rate</t>
+          <t>starting_isa</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.04</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>annual_isa_allowance</t>
+          <t>isa_growth_rate</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>40000</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>property_sale</t>
+          <t>annual_isa_allowance</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>350000</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>property_sale_age</t>
+          <t>property_sale</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>67</v>
+        <v>350000</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>state_pension_full</t>
+          <t>property_sale_age</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>12548</v>
+        <v>67</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>current_calendar_year</t>
+          <t>state_pension_full</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>2026</v>
+        <v>12548</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>state_pension_growth</t>
+          <t>current_calendar_year</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0.035</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>spending_phase_1</t>
+          <t>state_pension_growth</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>35000</v>
+        <v>0.035</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>spending_phase_2</t>
+          <t>spending_phase_1</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>32000</v>
+        <v>35000</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>spending_phase_3</t>
+          <t>spending_phase_2</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>28000</v>
+        <v>32000</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>phase_1_end_age</t>
+          <t>spending_phase_3</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>69</v>
+        <v>28000</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>phase_2_end_age</t>
+          <t>phase_1_end_age</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>79</v>
+        <v>69</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>inflation_rate</t>
+          <t>phase_2_end_age</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>0.025</v>
+        <v>79</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>inflation_link_spending</t>
-        </is>
-      </c>
-      <c r="B36" t="b">
-        <v>1</v>
+          <t>inflation_rate</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>0.025</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>inflation_link_tax</t>
+          <t>inflation_link_spending</t>
         </is>
       </c>
       <c r="B37" t="b">
@@ -909,15 +911,25 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>inflation_link_isa</t>
+          <t>inflation_link_tax</t>
         </is>
       </c>
       <c r="B38" t="b">
         <v>1</v>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>inflation_link_isa</t>
+        </is>
+      </c>
+      <c r="B39" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B38"/>
+  <autoFilter ref="A1:B39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1027,13 +1039,13 @@
         <v>26400</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>34357.5</v>
+        <v>40195</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>4357.5</v>
+        <v>5525</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>30000</v>
+        <v>34670</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>0</v>
@@ -1062,19 +1074,19 @@
         <v>2028</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>652042.5</v>
+        <v>646205</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>26081.7</v>
+        <v>25848.2</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>34357.5</v>
+        <v>40182.62</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>4357.5</v>
+        <v>5522.52</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>30000</v>
+        <v>34660.1</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>0</v>
@@ -1103,19 +1115,19 @@
         <v>2029</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>643766.7</v>
+        <v>631870.58</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>25750.67</v>
+        <v>25274.82</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>34357.5</v>
+        <v>40169.87</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>4357.5</v>
+        <v>5519.97</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>30000</v>
+        <v>34649.9</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>0</v>
@@ -1144,19 +1156,19 @@
         <v>2030</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>635159.87</v>
+        <v>616975.53</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>25406.39</v>
+        <v>24679.02</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>34357.5</v>
+        <v>40156.75</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>4357.5</v>
+        <v>5517.35</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>30000</v>
+        <v>34639.4</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>0</v>
@@ -1185,10 +1197,10 @@
         <v>2031</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>626208.76</v>
+        <v>601497.8</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>25048.35</v>
+        <v>24059.91</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>27595.22</v>
@@ -1226,10 +1238,10 @@
         <v>2032</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>623661.89</v>
+        <v>597962.5</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>24946.48</v>
+        <v>23918.5</v>
       </c>
       <c r="E7" s="2" t="n">
         <v>27142.12</v>
@@ -1267,10 +1279,10 @@
         <v>2033</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>621466.25</v>
+        <v>594738.88</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>24858.65</v>
+        <v>23789.56</v>
       </c>
       <c r="E8" s="2" t="n">
         <v>9871.059999999999</v>
@@ -1308,10 +1320,10 @@
         <v>2034</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>636453.84</v>
+        <v>608657.37</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>25458.15</v>
+        <v>24346.29</v>
       </c>
       <c r="E9" s="2" t="n">
         <v>5047.75</v>
@@ -1349,10 +1361,10 @@
         <v>2035</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>656864.24</v>
+        <v>627955.92</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>26274.57</v>
+        <v>25118.24</v>
       </c>
       <c r="E10" s="2" t="n">
         <v>3936.94</v>
@@ -1390,10 +1402,10 @@
         <v>2036</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>679201.87</v>
+        <v>649137.21</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>27168.07</v>
+        <v>25965.49</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>2787.32</v>
@@ -1431,10 +1443,10 @@
         <v>2037</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>703582.63</v>
+        <v>672315.38</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>28143.31</v>
+        <v>26892.62</v>
       </c>
       <c r="E12" s="2" t="n">
         <v>1597.56</v>
@@ -1472,10 +1484,10 @@
         <v>2038</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>730128.37</v>
+        <v>697610.4399999999</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>29205.13</v>
+        <v>27904.42</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>848.64</v>
@@ -1513,10 +1525,10 @@
         <v>2039</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>758484.87</v>
+        <v>724666.21</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>30339.39</v>
+        <v>28986.65</v>
       </c>
       <c r="E14" s="2" t="n">
         <v>988.33</v>
@@ -1554,10 +1566,10 @@
         <v>2040</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>787835.9300000001</v>
+        <v>752664.53</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>31513.44</v>
+        <v>30106.58</v>
       </c>
       <c r="E15" s="2" t="n">
         <v>1132.91</v>
@@ -1595,10 +1607,10 @@
         <v>2041</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>818216.46</v>
+        <v>781638.2</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>32728.66</v>
+        <v>31265.53</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>1282.55</v>
@@ -1636,10 +1648,10 @@
         <v>2042</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>849662.5699999999</v>
+        <v>811621.1800000001</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>33986.5</v>
+        <v>32464.85</v>
       </c>
       <c r="E17" s="2" t="n">
         <v>1437.42</v>
@@ -1677,10 +1689,10 @@
         <v>2043</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>882211.65</v>
+        <v>842648.61</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>35288.47</v>
+        <v>33705.94</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>1597.72</v>
@@ -1718,10 +1730,10 @@
         <v>2044</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>915902.4</v>
+        <v>874756.83</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>36636.1</v>
+        <v>34990.27</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>1763.63</v>
@@ -1759,10 +1771,10 @@
         <v>2045</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>950774.86</v>
+        <v>907983.48</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>38030.99</v>
+        <v>36319.34</v>
       </c>
       <c r="E20" s="2" t="n">
         <v>1935.34</v>
@@ -1800,10 +1812,10 @@
         <v>2046</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>986870.52</v>
+        <v>942367.48</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>39474.82</v>
+        <v>37694.7</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>2113.07</v>
@@ -1841,10 +1853,10 @@
         <v>2047</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1024232.27</v>
+        <v>977949.11</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>40969.29</v>
+        <v>39117.96</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>2297.01</v>
@@ -1882,10 +1894,10 @@
         <v>2048</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>1062904.55</v>
+        <v>1014770.06</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>42516.18</v>
+        <v>40590.8</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>2487.4</v>
@@ -1923,10 +1935,10 @@
         <v>2049</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1102933.33</v>
+        <v>1052873.46</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>44117.33</v>
+        <v>42114.94</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>2684.44</v>
@@ -1964,10 +1976,10 @@
         <v>2050</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>1144366.22</v>
+        <v>1092303.96</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>45774.65</v>
+        <v>43692.16</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>2888.39</v>
@@ -2005,10 +2017,10 @@
         <v>2051</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>1187252.48</v>
+        <v>1133107.73</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>47490.1</v>
+        <v>45324.31</v>
       </c>
       <c r="E26" s="2" t="n">
         <v>3099.47</v>
@@ -2046,10 +2058,10 @@
         <v>2052</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>1231643.11</v>
+        <v>1175332.57</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>49265.72</v>
+        <v>47013.3</v>
       </c>
       <c r="E27" s="2" t="n">
         <v>3317.94</v>
@@ -2087,10 +2099,10 @@
         <v>2053</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>1277590.9</v>
+        <v>1219027.93</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>51103.64</v>
+        <v>48761.12</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>3544.05</v>
@@ -2128,10 +2140,10 @@
         <v>2054</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>1325150.48</v>
+        <v>1264245</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>53006.02</v>
+        <v>50569.8</v>
       </c>
       <c r="E29" s="2" t="n">
         <v>3778.08</v>

</xml_diff>

<commit_message>
v0.6.0 - Introduce Optimisation Engine and structured planner workflow
</commit_message>
<xml_diff>
--- a/RetirementPlanner.xlsx
+++ b/RetirementPlanner.xlsx
@@ -483,7 +483,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>1311036.72</v>
+        <v>1789412.61</v>
       </c>
     </row>
     <row r="7">
@@ -1039,13 +1039,13 @@
         <v>26400</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>40195</v>
+        <v>12570</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>5525</v>
+        <v>0</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>34670</v>
+        <v>12570</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>0</v>
@@ -1074,19 +1074,19 @@
         <v>2028</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>646205</v>
+        <v>673830</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>25848.2</v>
+        <v>26953.2</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>40182.62</v>
+        <v>12570</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>5522.52</v>
+        <v>0</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>34660.1</v>
+        <v>12570</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>0</v>
@@ -1115,19 +1115,19 @@
         <v>2029</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>631870.58</v>
+        <v>688213.2</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>25274.82</v>
+        <v>27528.53</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>40169.87</v>
+        <v>12570</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>5519.97</v>
+        <v>0</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>34649.9</v>
+        <v>12570</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>0</v>
@@ -1156,19 +1156,19 @@
         <v>2030</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>616975.53</v>
+        <v>703171.73</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>24679.02</v>
+        <v>28126.87</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>40156.75</v>
+        <v>12570</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>5517.35</v>
+        <v>0</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>34639.4</v>
+        <v>12570</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>0</v>
@@ -1197,19 +1197,19 @@
         <v>2031</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>601497.8</v>
+        <v>718728.6</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>24059.91</v>
+        <v>28749.14</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>27595.22</v>
+        <v>22</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>5514.64</v>
+        <v>0</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>22080.58</v>
+        <v>22</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>12548</v>
@@ -1238,19 +1238,19 @@
         <v>2032</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>597962.5</v>
+        <v>747455.74</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>23918.5</v>
+        <v>29898.23</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>27142.12</v>
+        <v>104.29</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>5511.86</v>
+        <v>104.29</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>21630.26</v>
+        <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>12987.18</v>
@@ -1279,19 +1279,19 @@
         <v>2033</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>594738.88</v>
+        <v>777249.6800000001</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>23789.56</v>
+        <v>31089.99</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>9871.059999999999</v>
+        <v>217.93</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>2148.56</v>
+        <v>217.93</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>7722.5</v>
+        <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>13441.73</v>
@@ -1320,19 +1320,19 @@
         <v>2034</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>608657.37</v>
+        <v>808121.74</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>24346.29</v>
+        <v>32324.87</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>5047.75</v>
+        <v>335.55</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>1277.99</v>
+        <v>335.55</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>3769.76</v>
+        <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>13912.19</v>
@@ -1361,19 +1361,19 @@
         <v>2035</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>627955.92</v>
+        <v>840111.0600000001</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>25118.24</v>
+        <v>33604.44</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>3936.94</v>
+        <v>457.28</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>1153.21</v>
+        <v>457.28</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>2783.73</v>
+        <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
         <v>14399.12</v>
@@ -1402,19 +1402,19 @@
         <v>2036</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>649137.21</v>
+        <v>873258.22</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>25965.49</v>
+        <v>34930.33</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>2787.32</v>
+        <v>583.27</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>1024.08</v>
+        <v>583.27</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>1763.24</v>
+        <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>14903.09</v>
@@ -1443,19 +1443,19 @@
         <v>2037</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>672315.38</v>
+        <v>907605.28</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>26892.62</v>
+        <v>36304.21</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>1597.56</v>
+        <v>713.67</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>890.45</v>
+        <v>713.67</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>707.11</v>
+        <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>15424.7</v>
@@ -1484,10 +1484,10 @@
         <v>2038</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>697610.4399999999</v>
+        <v>943195.8199999999</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>27904.42</v>
+        <v>37727.83</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>848.64</v>
@@ -1525,10 +1525,10 @@
         <v>2039</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>724666.21</v>
+        <v>980075.01</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>28986.65</v>
+        <v>39203</v>
       </c>
       <c r="E14" s="2" t="n">
         <v>988.33</v>
@@ -1566,10 +1566,10 @@
         <v>2040</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>752664.53</v>
+        <v>1018289.68</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>30106.58</v>
+        <v>40731.59</v>
       </c>
       <c r="E15" s="2" t="n">
         <v>1132.91</v>
@@ -1607,10 +1607,10 @@
         <v>2041</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>781638.2</v>
+        <v>1057888.36</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>31265.53</v>
+        <v>42315.53</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>1282.55</v>
@@ -1648,10 +1648,10 @@
         <v>2042</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>811621.1800000001</v>
+        <v>1098921.34</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>32464.85</v>
+        <v>43956.85</v>
       </c>
       <c r="E17" s="2" t="n">
         <v>1437.42</v>
@@ -1689,10 +1689,10 @@
         <v>2043</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>842648.61</v>
+        <v>1141440.78</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>33705.94</v>
+        <v>45657.63</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>1597.72</v>
@@ -1730,10 +1730,10 @@
         <v>2044</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>874756.83</v>
+        <v>1185500.69</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>34990.27</v>
+        <v>47420.03</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>1763.63</v>
@@ -1771,10 +1771,10 @@
         <v>2045</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>907983.48</v>
+        <v>1231157.09</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>36319.34</v>
+        <v>49246.28</v>
       </c>
       <c r="E20" s="2" t="n">
         <v>1935.34</v>
@@ -1812,10 +1812,10 @@
         <v>2046</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>942367.48</v>
+        <v>1278468.03</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>37694.7</v>
+        <v>51138.72</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>2113.07</v>
@@ -1853,10 +1853,10 @@
         <v>2047</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>977949.11</v>
+        <v>1327493.68</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>39117.96</v>
+        <v>53099.75</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>2297.01</v>
@@ -1894,10 +1894,10 @@
         <v>2048</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>1014770.06</v>
+        <v>1378296.42</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>40590.8</v>
+        <v>55131.86</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>2487.4</v>
@@ -1935,10 +1935,10 @@
         <v>2049</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1052873.46</v>
+        <v>1430940.88</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>42114.94</v>
+        <v>57237.64</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>2684.44</v>
@@ -1976,10 +1976,10 @@
         <v>2050</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>1092303.96</v>
+        <v>1485494.07</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>43692.16</v>
+        <v>59419.76</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>2888.39</v>
@@ -2017,10 +2017,10 @@
         <v>2051</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>1133107.73</v>
+        <v>1542025.44</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>45324.31</v>
+        <v>61681.02</v>
       </c>
       <c r="E26" s="2" t="n">
         <v>3099.47</v>
@@ -2058,10 +2058,10 @@
         <v>2052</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>1175332.57</v>
+        <v>1600606.99</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>47013.3</v>
+        <v>64024.28</v>
       </c>
       <c r="E27" s="2" t="n">
         <v>3317.94</v>
@@ -2099,10 +2099,10 @@
         <v>2053</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>1219027.93</v>
+        <v>1661313.33</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>48761.12</v>
+        <v>66452.53</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>3544.05</v>
@@ -2140,10 +2140,10 @@
         <v>2054</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>1264245</v>
+        <v>1724221.81</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>50569.8</v>
+        <v>68968.87</v>
       </c>
       <c r="E29" s="2" t="n">
         <v>3778.08</v>

</xml_diff>

<commit_message>
RC2-P002 Add regression test framework
</commit_message>
<xml_diff>
--- a/RetirementPlanner.xlsx
+++ b/RetirementPlanner.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Charts" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Assumptions'!$A$1:$B$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Assumptions'!$A$1:$B$42</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Cash Flow'!$A$1:$M$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -483,7 +483,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>1789412.61</v>
+        <v>1311036.72</v>
       </c>
     </row>
     <row r="7">
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B39"/>
+  <dimension ref="A1:B42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -751,185 +751,215 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>savings_interest</t>
+          <t>expected_return</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.035</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>starting_isa</t>
+          <t>investment_volatility</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>50000</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>isa_growth_rate</t>
+          <t>inflation_volatility</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0.04</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>annual_isa_allowance</t>
+          <t>savings_interest</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>40000</v>
+        <v>0.035</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>property_sale</t>
+          <t>starting_isa</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>350000</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>property_sale_age</t>
+          <t>isa_growth_rate</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>67</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>state_pension_full</t>
+          <t>annual_isa_allowance</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>12548</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>current_calendar_year</t>
+          <t>property_sale</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>2026</v>
+        <v>350000</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>state_pension_growth</t>
+          <t>property_sale_age</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>0.035</v>
+        <v>67</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>spending_phase_1</t>
+          <t>state_pension_full</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>35000</v>
+        <v>12548</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>spending_phase_2</t>
+          <t>current_calendar_year</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>32000</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>spending_phase_3</t>
+          <t>state_pension_growth</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>28000</v>
+        <v>0.035</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>phase_1_end_age</t>
+          <t>spending_phase_1</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>69</v>
+        <v>35000</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>phase_2_end_age</t>
+          <t>spending_phase_2</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>79</v>
+        <v>32000</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>inflation_rate</t>
+          <t>spending_phase_3</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0.025</v>
+        <v>28000</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>inflation_link_spending</t>
-        </is>
-      </c>
-      <c r="B37" t="b">
-        <v>1</v>
+          <t>phase_1_end_age</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>69</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>inflation_link_tax</t>
-        </is>
-      </c>
-      <c r="B38" t="b">
-        <v>1</v>
+          <t>phase_2_end_age</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>79</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>inflation_rate</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>0.025</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>inflation_link_spending</t>
+        </is>
+      </c>
+      <c r="B40" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>inflation_link_tax</t>
+        </is>
+      </c>
+      <c r="B41" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
           <t>inflation_link_isa</t>
         </is>
       </c>
-      <c r="B39" t="b">
+      <c r="B42" t="b">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B39"/>
+  <autoFilter ref="A1:B42"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1039,13 +1069,13 @@
         <v>26400</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>12570</v>
+        <v>40195</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0</v>
+        <v>5525</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>12570</v>
+        <v>34670</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>0</v>
@@ -1074,19 +1104,19 @@
         <v>2028</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>673830</v>
+        <v>646205</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>26953.2</v>
+        <v>25848.2</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>12570</v>
+        <v>40182.62</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0</v>
+        <v>5522.52</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>12570</v>
+        <v>34660.1</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>0</v>
@@ -1115,19 +1145,19 @@
         <v>2029</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>688213.2</v>
+        <v>631870.58</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>27528.53</v>
+        <v>25274.82</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>12570</v>
+        <v>40169.87</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0</v>
+        <v>5519.97</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>12570</v>
+        <v>34649.9</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>0</v>
@@ -1156,19 +1186,19 @@
         <v>2030</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>703171.73</v>
+        <v>616975.53</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>28126.87</v>
+        <v>24679.02</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>12570</v>
+        <v>40156.75</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0</v>
+        <v>5517.35</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>12570</v>
+        <v>34639.4</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>0</v>
@@ -1197,19 +1227,19 @@
         <v>2031</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>718728.6</v>
+        <v>601497.8</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>28749.14</v>
+        <v>24059.91</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>22</v>
+        <v>27595.22</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0</v>
+        <v>5514.64</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>22</v>
+        <v>22080.58</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>12548</v>
@@ -1238,19 +1268,19 @@
         <v>2032</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>747455.74</v>
+        <v>597962.5</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>29898.23</v>
+        <v>23918.5</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>104.29</v>
+        <v>27142.12</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>104.29</v>
+        <v>5511.86</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>0</v>
+        <v>21630.26</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>12987.18</v>
@@ -1279,19 +1309,19 @@
         <v>2033</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>777249.6800000001</v>
+        <v>594738.88</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>31089.99</v>
+        <v>23789.56</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>217.93</v>
+        <v>9871.059999999999</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>217.93</v>
+        <v>2148.56</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>0</v>
+        <v>7722.5</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>13441.73</v>
@@ -1320,19 +1350,19 @@
         <v>2034</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>808121.74</v>
+        <v>608657.37</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>32324.87</v>
+        <v>24346.29</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>335.55</v>
+        <v>5047.75</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>335.55</v>
+        <v>1277.99</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>0</v>
+        <v>3769.76</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>13912.19</v>
@@ -1361,19 +1391,19 @@
         <v>2035</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>840111.0600000001</v>
+        <v>627955.92</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>33604.44</v>
+        <v>25118.24</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>457.28</v>
+        <v>3936.94</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>457.28</v>
+        <v>1153.21</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>0</v>
+        <v>2783.73</v>
       </c>
       <c r="H10" s="2" t="n">
         <v>14399.12</v>
@@ -1402,19 +1432,19 @@
         <v>2036</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>873258.22</v>
+        <v>649137.21</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>34930.33</v>
+        <v>25965.49</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>583.27</v>
+        <v>2787.32</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>583.27</v>
+        <v>1024.08</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>0</v>
+        <v>1763.24</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>14903.09</v>
@@ -1443,19 +1473,19 @@
         <v>2037</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>907605.28</v>
+        <v>672315.38</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>36304.21</v>
+        <v>26892.62</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>713.67</v>
+        <v>1597.56</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>713.67</v>
+        <v>890.45</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>0</v>
+        <v>707.11</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>15424.7</v>
@@ -1484,10 +1514,10 @@
         <v>2038</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>943195.8199999999</v>
+        <v>697610.4399999999</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>37727.83</v>
+        <v>27904.42</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>848.64</v>
@@ -1525,10 +1555,10 @@
         <v>2039</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>980075.01</v>
+        <v>724666.21</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>39203</v>
+        <v>28986.65</v>
       </c>
       <c r="E14" s="2" t="n">
         <v>988.33</v>
@@ -1566,10 +1596,10 @@
         <v>2040</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>1018289.68</v>
+        <v>752664.53</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>40731.59</v>
+        <v>30106.58</v>
       </c>
       <c r="E15" s="2" t="n">
         <v>1132.91</v>
@@ -1607,10 +1637,10 @@
         <v>2041</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1057888.36</v>
+        <v>781638.2</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>42315.53</v>
+        <v>31265.53</v>
       </c>
       <c r="E16" s="2" t="n">
         <v>1282.55</v>
@@ -1648,10 +1678,10 @@
         <v>2042</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>1098921.34</v>
+        <v>811621.1800000001</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>43956.85</v>
+        <v>32464.85</v>
       </c>
       <c r="E17" s="2" t="n">
         <v>1437.42</v>
@@ -1689,10 +1719,10 @@
         <v>2043</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1141440.78</v>
+        <v>842648.61</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>45657.63</v>
+        <v>33705.94</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>1597.72</v>
@@ -1730,10 +1760,10 @@
         <v>2044</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1185500.69</v>
+        <v>874756.83</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>47420.03</v>
+        <v>34990.27</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>1763.63</v>
@@ -1771,10 +1801,10 @@
         <v>2045</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1231157.09</v>
+        <v>907983.48</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>49246.28</v>
+        <v>36319.34</v>
       </c>
       <c r="E20" s="2" t="n">
         <v>1935.34</v>
@@ -1812,10 +1842,10 @@
         <v>2046</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1278468.03</v>
+        <v>942367.48</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>51138.72</v>
+        <v>37694.7</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>2113.07</v>
@@ -1853,10 +1883,10 @@
         <v>2047</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1327493.68</v>
+        <v>977949.11</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>53099.75</v>
+        <v>39117.96</v>
       </c>
       <c r="E22" s="2" t="n">
         <v>2297.01</v>
@@ -1894,10 +1924,10 @@
         <v>2048</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>1378296.42</v>
+        <v>1014770.06</v>
       </c>
       <c r="D23" s="2" t="n">
-        <v>55131.86</v>
+        <v>40590.8</v>
       </c>
       <c r="E23" s="2" t="n">
         <v>2487.4</v>
@@ -1935,10 +1965,10 @@
         <v>2049</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1430940.88</v>
+        <v>1052873.46</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>57237.64</v>
+        <v>42114.94</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>2684.44</v>
@@ -1976,10 +2006,10 @@
         <v>2050</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>1485494.07</v>
+        <v>1092303.96</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>59419.76</v>
+        <v>43692.16</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>2888.39</v>
@@ -2017,10 +2047,10 @@
         <v>2051</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>1542025.44</v>
+        <v>1133107.73</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>61681.02</v>
+        <v>45324.31</v>
       </c>
       <c r="E26" s="2" t="n">
         <v>3099.47</v>
@@ -2058,10 +2088,10 @@
         <v>2052</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>1600606.99</v>
+        <v>1175332.57</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>64024.28</v>
+        <v>47013.3</v>
       </c>
       <c r="E27" s="2" t="n">
         <v>3317.94</v>
@@ -2099,10 +2129,10 @@
         <v>2053</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>1661313.33</v>
+        <v>1219027.93</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>66452.53</v>
+        <v>48761.12</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>3544.05</v>
@@ -2140,10 +2170,10 @@
         <v>2054</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>1724221.81</v>
+        <v>1264245</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>68968.87</v>
+        <v>50569.8</v>
       </c>
       <c r="E29" s="2" t="n">
         <v>3778.08</v>

</xml_diff>